<commit_message>
Add Gunma to integrated Excel builds (sheet and location maps)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0193CqecewNJBMTKaQ1KF3XN
</commit_message>
<xml_diff>
--- a/research/自治体_公共交通計画_環境基本計画_終期一覧_2026-09.xlsx
+++ b/research/自治体_公共交通計画_環境基本計画_終期一覧_2026-09.xlsx
@@ -16,6 +16,7 @@
     <sheet name="福島県" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="茨城県" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="栃木県" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="群馬県" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="TGT_MIN">'集計・設定'!$C$4</definedName>
@@ -28,6 +29,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'福島県'!$A$3:$T$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'茨城県'!$A$3:$T$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'栃木県'!$A$3:$T$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'群馬県'!$A$3:$T$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -604,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -992,163 +994,198 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>群馬県</t>
+        </is>
+      </c>
+      <c r="C17" s="3">
+        <f>COUNTA('群馬県'!$C$4:$C$38)</f>
+        <v/>
+      </c>
+      <c r="D17" s="3">
+        <f>COUNTIF('群馬県'!$C$4:$C$38,"◎ 営業")</f>
+        <v/>
+      </c>
+      <c r="E17" s="3">
+        <f>COUNTIF('群馬県'!$C$4:$C$38,"△ 着手済・要確認")</f>
+        <v/>
+      </c>
+      <c r="F17" s="3">
+        <f>COUNTIF('群馬県'!$C$4:$C$38,"？ 期間要確認")</f>
+        <v/>
+      </c>
+      <c r="G17" s="3">
+        <f>COUNTIF('群馬県'!$C$4:$C$38,"✕ 対象外")</f>
+        <v/>
+      </c>
+      <c r="H17" s="3">
+        <f>COUNTIF('群馬県'!$S$4:$S$38,"未調査")</f>
+        <v/>
+      </c>
+      <c r="I17" s="3">
+        <f>COUNTIF('群馬県'!$S$4:$S$38,"交通のみ調査")+COUNTIF('群馬県'!$S$4:$S$38,"環境のみ調査")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C17" s="2">
-        <f>SUM(C9:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="2">
-        <f>SUM(D9:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="2">
-        <f>SUM(E9:E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="2">
-        <f>SUM(F9:F16)</f>
-        <v/>
-      </c>
-      <c r="G17" s="2">
-        <f>SUM(G9:G16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="2">
-        <f>SUM(H9:H16)</f>
-        <v/>
-      </c>
-      <c r="I17" s="2">
-        <f>SUM(I9:I16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="C18" s="2">
+        <f>SUM(C9:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="2">
+        <f>SUM(D9:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="2">
+        <f>SUM(E9:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="2">
+        <f>SUM(F9:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="2">
+        <f>SUM(G9:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="2">
+        <f>SUM(H9:H17)</f>
+        <v/>
+      </c>
+      <c r="I18" s="2">
+        <f>SUM(I9:I17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>■ 判定の見方</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>◎ 営業：どちらかの計画の終期が対象年度（初期値R9）で、次の計画の作業は見つかっていない</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>△ 着手済・要確認：終期は対象年度だが、次期計画の策定業務委託やパブコメをすでに確認済。委託先が決まっている可能性が高い</t>
+          <t>◎ 営業：どちらかの計画の終期が対象年度（初期値R9）で、次の計画の作業は見つかっていない</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>？ 期間要確認：終期がわからないため判定できない</t>
+          <t>△ 着手済・要確認：終期は対象年度だが、次期計画の策定業務委託やパブコメをすでに確認済。委託先が決まっている可能性が高い</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>✕ 対象外：終期が対象年度の外（R8以前は作成中または終了、R10以降は先）、または新計画を策定済</t>
+          <t>？ 期間要確認：終期がわからないため判定できない</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
+          <t>✕ 対象外：終期が対象年度の外（R8以前は作成中または終了、R10以降は先）、または新計画を策定済</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
           <t>－：その計画がない（環境基本計画を作っていない町村など）</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>■ 入力する列</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>各県シートの「終期(令和年度)」と「改定状況」（未確認／着手済／策定済／計画なし）を直すと、判定が自動で変わります。</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>「未確認」は、改定の動きが検索で見つからなかったという意味です。動きがないと確かめたわけではありません。</t>
+          <t>各県シートの「終期(令和年度)」と「改定状況」（未確認／着手済／策定済／計画なし）を直すと、判定が自動で変わります。</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
+          <t>「未確認」は、改定の動きが検索で見つからなかったという意味です。動きがないと確かめたわけではありません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
           <t>確度：確認済＝検索結果の本文に期間が書かれていた／推定＝策定時期などから推測（終期のセルは茶色の斜体）／不明＝確認できなかった</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr"/>
-    </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>■ 国交省一覧との照合（T列）</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>国土交通省「地域公共交通計画の作成状況一覧」（令和8年5月末時点）と照合。掲載＝計画作成済み、期間満了＝一覧で灰色（計画期間が満了）。一覧には計画期間の記載がないため、終期は各計画書で確認。</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
+          <t>国土交通省「地域公共交通計画の作成状況一覧」（令和8年5月末時点）と照合。掲載＝計画作成済み、期間満了＝一覧で灰色（計画期間が満了）。一覧には計画期間の記載がないため、終期は各計画書で確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
           <t>【当方未把握】＝一覧には計画があるが本調査で計画書を特定できていない／【当方は計画あり】＝本調査では計画を把握したが一覧に未掲載（旧法計画・最近の策定・名称違いの可能性）。</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr"/>
-    </row>
     <row r="35">
-      <c r="A35" s="7" t="inlineStr">
+      <c r="A35" s="8" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>■ 調査の方法と限界</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>【重要】検索回数に上限（1セッション200回）があるため、県によっては一部の市町村・計画を調べきれていません。「調査状況」列が「未調査」「交通のみ調査」の行は空欄・？になっていますが、計画がないという意味ではありません。</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>2026年9月30日時点でWeb検索して調べました。自治体サイトやPDFを直接開けない環境だったため、期間は検索結果の本文・要約から取っています。</t>
+          <t>【重要】検索回数に上限（1セッション200回）があるため、県によっては一部の市町村・計画を調べきれていません。「調査状況」列が「未調査」「交通のみ調査」の行は空欄・？になっていますが、計画がないという意味ではありません。</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>2026年9月30日時点でWeb検索して調べました。自治体サイトやPDFを直接開けない環境だったため、期間は検索結果の本文・要約から取っています。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>計画リンクはエビデンスとして検索結果に出たURLを載せています。営業に行く前に、リンク先の計画書で計画期間を確かめてください。特に「推定」「不明」の行は必ず確認してください。</t>
         </is>
@@ -1160,6 +1197,2984 @@
       <formula1>"7,8,9,10,11,12,13,14,15"</formula1>
     </dataValidation>
   </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="55" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>群馬県　地域公共交通計画・環境基本計画の終期一覧（2026年9月30日時点の調査）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9">
+        <f>"営業判定の対象：終期 R"&amp;TGT_MIN&amp;"〜R"&amp;TGT_MAX&amp;"年度 →◎（着手済は△、期間不明は？）。終期セルの色：緑＝対象年度／橙＝その翌年度（次の候補）。対象年度は「集計・設定」シートのC4・C5のプルダウンで切替。"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>市町村</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>営業判定</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>交通判定</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>環境判定</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>地域公共交通計画</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>交通 計画期間</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>交通 終期(令和年度)</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
+        <is>
+          <t>交通 確度</t>
+        </is>
+      </c>
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>交通 改定状況</t>
+        </is>
+      </c>
+      <c r="K3" s="10" t="inlineStr">
+        <is>
+          <t>交通 計画リンク（エビデンス）</t>
+        </is>
+      </c>
+      <c r="L3" s="10" t="inlineStr">
+        <is>
+          <t>環境基本計画</t>
+        </is>
+      </c>
+      <c r="M3" s="10" t="inlineStr">
+        <is>
+          <t>環境 計画期間</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
+          <t>環境 終期(令和年度)</t>
+        </is>
+      </c>
+      <c r="O3" s="10" t="inlineStr">
+        <is>
+          <t>環境 確度</t>
+        </is>
+      </c>
+      <c r="P3" s="10" t="inlineStr">
+        <is>
+          <t>環境 改定状況</t>
+        </is>
+      </c>
+      <c r="Q3" s="10" t="inlineStr">
+        <is>
+          <t>環境 計画リンク（エビデンス）</t>
+        </is>
+      </c>
+      <c r="R3" s="10" t="inlineStr">
+        <is>
+          <t>注釈（改定作業の状況など）</t>
+        </is>
+      </c>
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>調査状況</t>
+        </is>
+      </c>
+      <c r="T3" s="10" t="inlineStr">
+        <is>
+          <t>国交省一覧(R8.5末)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>前橋市</t>
+        </is>
+      </c>
+      <c r="C4" s="12">
+        <f>IF(OR(D4="◎",E4="◎"),"◎ 営業",IF(OR(D4="△",E4="△"),"△ 着手済・要確認",IF(OR(D4="？",E4="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D4" s="13">
+        <f>IF(J4="計画なし","－",IF(J4="策定済","✕",IF(H4="","？",IF(AND(H4&gt;=TGT_MIN,H4&lt;=TGT_MAX),IF(J4="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E4" s="13">
+        <f>IF(P4="計画なし","－",IF(P4="策定済","✕",IF(N4="","？",IF(AND(N4&gt;=TGT_MIN,N4&lt;=TGT_MAX),IF(P4="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>前橋市地域公共交通計画（次期）</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>R8〜R12</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.maebashi.gunma.jp/material/files/group/9/6keikakusouann7-2-4.pdf</t>
+        </is>
+      </c>
+      <c r="L4" s="11" t="inlineStr">
+        <is>
+          <t>前橋市環境基本計画（平成29年度改訂）</t>
+        </is>
+      </c>
+      <c r="M4" s="11" t="inlineStr">
+        <is>
+          <t>H30〜R9</t>
+        </is>
+      </c>
+      <c r="N4" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="O4" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P4" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="Q4" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.maebashi.gunma.jp/soshiki/kankyo/kankyoseisaku/gyomu/2_1/5/2718.html</t>
+        </is>
+      </c>
+      <c r="R4" s="11" t="inlineStr">
+        <is>
+          <t>交通：R3.6策定の現行計画がR7年度で目標年次を迎え、R8〜R12の次期計画を策定（t_urlは計画素案PDF、最終決定版URLは未確認）。環境：適用期間H30〜R9（2018〜2027）でR9終期。環境政策課ページの「前橋市環境基本計画改訂業務の実施事業者が決定」告知は、H29年度の前回改訂（仕様書の履行期限H30.3.30 https://www.city.maebashi.gunma.jp/material/files/group/46/siyosyo.pdf ）のものと判断。R8年度の次期計画の審議会諮問・委託は検索で確認できず（R6年度環境審議会でも諮問の記載なし https://www.city.maebashi.gunma.jp/soshiki/kankyo/kankyoseisaku/gyomu/5/1/43841.html ）。同時期に緑の基本計画改定支援業務（R8.10〜R10.3予定 https://www.city.maebashi.gunma.jp/material/files/group/67/siyousyoan.pdf ）・第八次総合計画策定支援（R8.4〜R10.3）が進行中。</t>
+        </is>
+      </c>
+      <c r="S4" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T4" s="11" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>高崎市</t>
+        </is>
+      </c>
+      <c r="C5" s="12">
+        <f>IF(OR(D5="◎",E5="◎"),"◎ 営業",IF(OR(D5="△",E5="△"),"△ 着手済・要確認",IF(OR(D5="？",E5="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D5" s="13">
+        <f>IF(J5="計画なし","－",IF(J5="策定済","✕",IF(H5="","？",IF(AND(H5&gt;=TGT_MIN,H5&lt;=TGT_MAX),IF(J5="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E5" s="13">
+        <f>IF(P5="計画なし","－",IF(P5="策定済","✕",IF(N5="","？",IF(AND(N5&gt;=TGT_MIN,N5&lt;=TGT_MAX),IF(P5="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F5" s="11" t="n"/>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="n"/>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="n"/>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>高崎市第4次環境基本計画</t>
+        </is>
+      </c>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>H30〜R9</t>
+        </is>
+      </c>
+      <c r="N5" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P5" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="Q5" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.takasaki.gunma.jp/page/3402.html</t>
+        </is>
+      </c>
+      <c r="R5" s="11" t="inlineStr">
+        <is>
+          <t>交通：市独自の地域公共交通計画は検索で確認できず（地域公共交通会議 https://www.city.takasaki.gunma.jp/page/59580.html はあり、ぐるりん等を運営）。環境：第4次2018〜2027年度でR9終期。環境審議会ページが2026.8.28更新 https://www.city.takasaki.gunma.jp/page/3275.html 、委員はR8.4〜R10.3任期で改選。次期計画の委託・諮問は未確認だが審議開始の可能性大、要注視。</t>
+        </is>
+      </c>
+      <c r="S5" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T5" s="11" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>桐生市</t>
+        </is>
+      </c>
+      <c r="C6" s="12">
+        <f>IF(OR(D6="◎",E6="◎"),"◎ 営業",IF(OR(D6="△",E6="△"),"△ 着手済・要確認",IF(OR(D6="？",E6="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D6" s="13">
+        <f>IF(J6="計画なし","－",IF(J6="策定済","✕",IF(H6="","？",IF(AND(H6&gt;=TGT_MIN,H6&lt;=TGT_MAX),IF(J6="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E6" s="13">
+        <f>IF(P6="計画なし","－",IF(P6="策定済","✕",IF(N6="","？",IF(AND(N6&gt;=TGT_MIN,N6&lt;=TGT_MAX),IF(P6="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>桐生市地域公共交通計画</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>R6〜R10</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.kiryu.lg.jp/_res/projects/default_project/_page_/001/024/200/tpplan2024.pdf</t>
+        </is>
+      </c>
+      <c r="L6" s="11" t="inlineStr">
+        <is>
+          <t>第3次桐生市環境基本計画</t>
+        </is>
+      </c>
+      <c r="M6" s="11" t="inlineStr">
+        <is>
+          <t>R3〜R12</t>
+        </is>
+      </c>
+      <c r="N6" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="O6" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P6" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="Q6" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.kiryu.lg.jp/shisei/keikaku/1018141/1002981.html</t>
+        </is>
+      </c>
+      <c r="R6" s="11" t="inlineStr">
+        <is>
+          <t>交通：R6.6策定、R6〜R10、上位に桐生市交通ビジョン（R15目途）。環境：R3〜R12の10年。環境先進都市将来構想を2025.3改定し2050年まで延長との記載あり（https://www.city.kiryu.lg.jp/_res/projects/default_project/_page_/001/000/874/kiryusinokankyo2025.pdf ）。</t>
+        </is>
+      </c>
+      <c r="S6" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T6" s="11" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>伊勢崎市</t>
+        </is>
+      </c>
+      <c r="C7" s="12">
+        <f>IF(OR(D7="◎",E7="◎"),"◎ 営業",IF(OR(D7="△",E7="△"),"△ 着手済・要確認",IF(OR(D7="？",E7="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D7" s="13">
+        <f>IF(J7="計画なし","－",IF(J7="策定済","✕",IF(H7="","？",IF(AND(H7&gt;=TGT_MIN,H7&lt;=TGT_MAX),IF(J7="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E7" s="13">
+        <f>IF(P7="計画なし","－",IF(P7="策定済","✕",IF(N7="","？",IF(AND(N7&gt;=TGT_MIN,N7&lt;=TGT_MAX),IF(P7="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>伊勢崎市地域公共交通計画（策定中）</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="n"/>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>着手済</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="n"/>
+      <c r="L7" s="11" t="inlineStr">
+        <is>
+          <t>第3次伊勢崎市環境基本計画</t>
+        </is>
+      </c>
+      <c r="M7" s="11" t="inlineStr">
+        <is>
+          <t>R7〜R16</t>
+        </is>
+      </c>
+      <c r="N7" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="O7" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P7" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="Q7" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.isesaki.lg.jp/material/files/group/29/dai3jikankyoukihonkeikaku.pdf</t>
+        </is>
+      </c>
+      <c r="R7" s="11" t="inlineStr">
+        <is>
+          <t>交通：現行の法定計画は確認できず。R7.7地域公共交通会議で計画策定に伴う法定協議会への移行を協議、R8.4に計画策定業務委託プロポーザル公告（R8.6頃選定、契約初年度R9.3まで） https://www.city.isesaki.lg.jp/sangyo_nyusatsu_kaihatsu/nyusatsu_keiyaku/proposal/23159.html 。環境：R7.3策定、R7〜R16の10年。</t>
+        </is>
+      </c>
+      <c r="S7" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T7" s="11" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>太田市</t>
+        </is>
+      </c>
+      <c r="C8" s="12">
+        <f>IF(OR(D8="◎",E8="◎"),"◎ 営業",IF(OR(D8="△",E8="△"),"△ 着手済・要確認",IF(OR(D8="？",E8="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D8" s="13">
+        <f>IF(J8="計画なし","－",IF(J8="策定済","✕",IF(H8="","？",IF(AND(H8&gt;=TGT_MIN,H8&lt;=TGT_MAX),IF(J8="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E8" s="13">
+        <f>IF(P8="計画なし","－",IF(P8="策定済","✕",IF(N8="","？",IF(AND(N8&gt;=TGT_MIN,N8&lt;=TGT_MAX),IF(P8="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>太田市地域公共交通計画（策定中）</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="n"/>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>着手済</t>
+        </is>
+      </c>
+      <c r="K8" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.ota.gunma.jp/page/1051226.html</t>
+        </is>
+      </c>
+      <c r="L8" s="11" t="inlineStr">
+        <is>
+          <t>第2次太田市環境基本計画（2022改定版）</t>
+        </is>
+      </c>
+      <c r="M8" s="11" t="inlineStr">
+        <is>
+          <t>H29〜R8（改定版R4〜R8）</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="O8" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t>着手済</t>
+        </is>
+      </c>
+      <c r="Q8" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.ota.gunma.jp/uploaded/attachment/2236.pdf</t>
+        </is>
+      </c>
+      <c r="R8" s="11" t="inlineStr">
+        <is>
+          <t>交通：前身の太田市地域公共交通網形成計画はH29〜R6（H36）で終了 https://www.city.ota.gunma.jp/page/2288.html 。後継の地域公共交通計画策定支援業務委託プロポーザルの審査結果を公表（t_url）、策定作業中。環境：2026年度で終期、第3次計画策定のワークショップを2026.8.3・8.28に開催 https://www.city.ota.gunma.jp/page/1059507.html 。</t>
+        </is>
+      </c>
+      <c r="S8" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T8" s="11" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>沼田市</t>
+        </is>
+      </c>
+      <c r="C9" s="12">
+        <f>IF(OR(D9="◎",E9="◎"),"◎ 営業",IF(OR(D9="△",E9="△"),"△ 着手済・要確認",IF(OR(D9="？",E9="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D9" s="13">
+        <f>IF(J9="計画なし","－",IF(J9="策定済","✕",IF(H9="","？",IF(AND(H9&gt;=TGT_MIN,H9&lt;=TGT_MAX),IF(J9="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E9" s="13">
+        <f>IF(P9="計画なし","－",IF(P9="策定済","✕",IF(N9="","？",IF(AND(N9&gt;=TGT_MIN,N9&lt;=TGT_MAX),IF(P9="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>沼田市地域公共交通計画</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>R6〜R9</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>推定</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="K9" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.numata.gunma.jp/life/kotsu/bus/1014138.html</t>
+        </is>
+      </c>
+      <c r="L9" s="11" t="inlineStr">
+        <is>
+          <t>第3次沼田市環境基本計画</t>
+        </is>
+      </c>
+      <c r="M9" s="11" t="inlineStr">
+        <is>
+          <t>R7〜（10年、終期未確認）</t>
+        </is>
+      </c>
+      <c r="N9" s="16" t="n"/>
+      <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t>推定</t>
+        </is>
+      </c>
+      <c r="P9" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="Q9" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.numata.gunma.jp/shisei/keikaku/keikaku/1016056.html</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>交通：R6.3策定。協議会資料（令和6年度第3回、R7.1）に「令和6年3月～令和10年3月」の記載あり https://www.city.numata.gunma.jp/_res/projects/default_project/_page_/001/014/867/numachikoshiryo.pdf （補助事業欄の記載で計画本文では未確認のため推定）。R8年度第1回協議会でR9年度確保維持事業の計画認定申請を協議 https://www.city.numata.gunma.jp/life/kotsu/bus/1014867.html 。次期計画の着手は未確認。環境：第二次（H27〜R6）満了を受け第3次を策定、今後10年（R7〜R16推定）。</t>
+        </is>
+      </c>
+      <c r="S9" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>館林市</t>
+        </is>
+      </c>
+      <c r="C10" s="12">
+        <f>IF(OR(D10="◎",E10="◎"),"◎ 営業",IF(OR(D10="△",E10="△"),"△ 着手済・要確認",IF(OR(D10="？",E10="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D10" s="13">
+        <f>IF(J10="計画なし","－",IF(J10="策定済","✕",IF(H10="","？",IF(AND(H10&gt;=TGT_MIN,H10&lt;=TGT_MAX),IF(J10="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E10" s="13">
+        <f>IF(P10="計画なし","－",IF(P10="策定済","✕",IF(N10="","？",IF(AND(N10&gt;=TGT_MIN,N10&lt;=TGT_MAX),IF(P10="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>第2次館林都市圏地域公共交通計画（1市4町共同）</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>R8〜R12</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>推定</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="K10" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.tatebayashi.gunma.jp/s015/shisei/040/020tatebayashitoshikenchiikikoukyoukoutukeikaku/2ndtatebayashitoshikentiikikoukyoukoutukeikaku.pdf</t>
+        </is>
+      </c>
+      <c r="L10" s="11" t="inlineStr">
+        <is>
+          <t>第三次館林市環境基本計画</t>
+        </is>
+      </c>
+      <c r="M10" s="11" t="inlineStr">
+        <is>
+          <t>R2〜R11</t>
+        </is>
+      </c>
+      <c r="N10" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="O10" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P10" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="Q10" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.tatebayashi.gunma.jp/s024/kurashi/120/080/020/kankyo-keikaku.pdf</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>交通：第2次館林都市圏地域公共交通計画（館林市・板倉町・明和町・千代田町・邑楽町の1市4町共同）。前計画R3〜R7の後継、パブコメR7.12.22〜R8.1.16、目標年次R12（期間R8〜R12は推定）。環境：R2〜R11の10年、R6年度中間見直し済。</t>
+        </is>
+      </c>
+      <c r="S10" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>渋川市</t>
+        </is>
+      </c>
+      <c r="C11" s="12">
+        <f>IF(OR(D11="◎",E11="◎"),"◎ 営業",IF(OR(D11="△",E11="△"),"△ 着手済・要確認",IF(OR(D11="？",E11="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D11" s="13">
+        <f>IF(J11="計画なし","－",IF(J11="策定済","✕",IF(H11="","？",IF(AND(H11&gt;=TGT_MIN,H11&lt;=TGT_MAX),IF(J11="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E11" s="13">
+        <f>IF(P11="計画なし","－",IF(P11="策定済","✕",IF(N11="","？",IF(AND(N11&gt;=TGT_MIN,N11&lt;=TGT_MAX),IF(P11="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>渋川市地域公共交通計画（R6.3一部変更 アフターコロナ編）</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>R3〜R7</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="K11" s="14" t="inlineStr">
+        <is>
+          <t>http://www.city.shibukawa.lg.jp/shisei/000259/000269/p006726.html</t>
+        </is>
+      </c>
+      <c r="L11" s="11" t="inlineStr">
+        <is>
+          <t>第2次渋川市環境基本計画（2024-2028）</t>
+        </is>
+      </c>
+      <c r="M11" s="11" t="inlineStr">
+        <is>
+          <t>R6〜R10</t>
+        </is>
+      </c>
+      <c r="N11" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="O11" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P11" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="Q11" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.shibukawa.lg.jp/kurashi/gomi/kankyoseisaku/p006733.html</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>交通：R3〜R7で期間満了、後継計画は検索で未確認。環境：当初R1〜R10の10年計画をR5年度に見直し、R6〜R10の5年計画に。</t>
+        </is>
+      </c>
+      <c r="S11" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>藤岡市</t>
+        </is>
+      </c>
+      <c r="C12" s="12">
+        <f>IF(OR(D12="◎",E12="◎"),"◎ 営業",IF(OR(D12="△",E12="△"),"△ 着手済・要確認",IF(OR(D12="？",E12="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D12" s="13">
+        <f>IF(J12="計画なし","－",IF(J12="策定済","✕",IF(H12="","？",IF(AND(H12&gt;=TGT_MIN,H12&lt;=TGT_MAX),IF(J12="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E12" s="13">
+        <f>IF(P12="計画なし","－",IF(P12="策定済","✕",IF(N12="","？",IF(AND(N12&gt;=TGT_MIN,N12&lt;=TGT_MAX),IF(P12="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="n"/>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K12" s="11" t="n"/>
+      <c r="L12" s="11" t="inlineStr">
+        <is>
+          <t>第3次藤岡市環境基本計画（R5.3改訂版）</t>
+        </is>
+      </c>
+      <c r="M12" s="11" t="inlineStr">
+        <is>
+          <t>R1〜R10</t>
+        </is>
+      </c>
+      <c r="N12" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="O12" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P12" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="Q12" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.fujioka.gunma.jp/material/files/group/21/gaiyouR05.pdf</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>交通：市独自の地域公共交通計画は検索で確認できず（路線バス「めぐるん」、前橋工科大学へのバス路線再編支援業務の調査報告書あり https://www.city.fujioka.gunma.jp/soshiki/somubu/chiikianzen/2/1/9133.html ）。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。環境：2019〜2028年度の10年、R5.3に前倒し見直し。e_urlは環境事業概要（計画書本体URLは未確認）。</t>
+        </is>
+      </c>
+      <c r="S12" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T12" s="11" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>富岡市</t>
+        </is>
+      </c>
+      <c r="C13" s="12">
+        <f>IF(OR(D13="◎",E13="◎"),"◎ 営業",IF(OR(D13="△",E13="△"),"△ 着手済・要確認",IF(OR(D13="？",E13="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D13" s="13">
+        <f>IF(J13="計画なし","－",IF(J13="策定済","✕",IF(H13="","？",IF(AND(H13&gt;=TGT_MIN,H13&lt;=TGT_MAX),IF(J13="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E13" s="13">
+        <f>IF(P13="計画なし","－",IF(P13="策定済","✕",IF(N13="","？",IF(AND(N13&gt;=TGT_MIN,N13&lt;=TGT_MAX),IF(P13="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>富岡市地域公共交通網形成計画（富岡市 都市と交通のマスタープラン内）</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>R2〜R6</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.tomioka.lg.jp/www/contents/1597279234959/simple/03_koukyoukoutsuu.pdf</t>
+        </is>
+      </c>
+      <c r="L13" s="11" t="inlineStr">
+        <is>
+          <t>第3次富岡市環境基本計画</t>
+        </is>
+      </c>
+      <c r="M13" s="11" t="inlineStr">
+        <is>
+          <t>R4〜R13</t>
+        </is>
+      </c>
+      <c r="N13" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="O13" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P13" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="Q13" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.tomioka.lg.jp/www/section/1000000000100/index.html</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr">
+        <is>
+          <t>交通：網形成計画2020〜2024年度で期間満了、後継の地域公共交通計画は検索で確認できず。環境：総合計画後期基本計画の関連計画一覧で期間R4〜R13、R4.3パブコメ結果公表（e_urlは環境政策課ページ）。</t>
+        </is>
+      </c>
+      <c r="S13" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T13" s="11" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>安中市</t>
+        </is>
+      </c>
+      <c r="C14" s="12">
+        <f>IF(OR(D14="◎",E14="◎"),"◎ 営業",IF(OR(D14="△",E14="△"),"△ 着手済・要確認",IF(OR(D14="？",E14="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D14" s="13">
+        <f>IF(J14="計画なし","－",IF(J14="策定済","✕",IF(H14="","？",IF(AND(H14&gt;=TGT_MIN,H14&lt;=TGT_MAX),IF(J14="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E14" s="13">
+        <f>IF(P14="計画なし","－",IF(P14="策定済","✕",IF(N14="","？",IF(AND(N14&gt;=TGT_MIN,N14&lt;=TGT_MAX),IF(P14="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>安中市地域公共交通計画</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>R8〜R12</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.annaka.lg.jp/page/17203.html</t>
+        </is>
+      </c>
+      <c r="L14" s="11" t="inlineStr">
+        <is>
+          <t>安中市環境基本計画2026</t>
+        </is>
+      </c>
+      <c r="M14" s="11" t="inlineStr">
+        <is>
+          <t>R8〜R17</t>
+        </is>
+      </c>
+      <c r="N14" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="O14" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P14" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="Q14" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.annaka.lg.jp/page/1015.html</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr">
+        <is>
+          <t>交通：2026.3.9策定公表、R8〜R12。環境：R8〜R17の新計画（市の計画一覧ページで期間確認）。</t>
+        </is>
+      </c>
+      <c r="S14" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T14" s="11" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>みどり市</t>
+        </is>
+      </c>
+      <c r="C15" s="12">
+        <f>IF(OR(D15="◎",E15="◎"),"◎ 営業",IF(OR(D15="△",E15="△"),"△ 着手済・要確認",IF(OR(D15="？",E15="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D15" s="13">
+        <f>IF(J15="計画なし","－",IF(J15="策定済","✕",IF(H15="","？",IF(AND(H15&gt;=TGT_MIN,H15&lt;=TGT_MAX),IF(J15="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E15" s="13">
+        <f>IF(P15="計画なし","－",IF(P15="策定済","✕",IF(N15="","？",IF(AND(N15&gt;=TGT_MIN,N15&lt;=TGT_MAX),IF(P15="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>みどり市地域公共交通計画</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>R8〜R12</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="K15" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.midori.gunma.jp/_res/projects/default_project/_page_/001/009/285/keikaku.pdf</t>
+        </is>
+      </c>
+      <c r="L15" s="11" t="inlineStr">
+        <is>
+          <t>第2次みどり市環境基本計画・後期基本計画</t>
+        </is>
+      </c>
+      <c r="M15" s="11" t="inlineStr">
+        <is>
+          <t>R5〜R9</t>
+        </is>
+      </c>
+      <c r="N15" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="O15" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P15" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="Q15" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.midori.gunma.jp/_res/projects/default_project/_page_/001/005/834/sdgs_midori_202504kaisei.pdf</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="inlineStr">
+        <is>
+          <t>交通：R6〜R7の2か年で策定支援業務（プロポーザル https://www.city.midori.gunma.jp/kurashi/1001625/1006056/1006059.html ）、R8〜R12。環境：後期基本計画2023〜2027年度でR9終期（期間はSDGs未来都市計画の記載で確認、計画書本体URLは未確認）。次期計画の着手は未確認。2050年みどり5つのゼロ宣言。</t>
+        </is>
+      </c>
+      <c r="S15" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T15" s="11" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>榛東村</t>
+        </is>
+      </c>
+      <c r="C16" s="12">
+        <f>IF(OR(D16="◎",E16="◎"),"◎ 営業",IF(OR(D16="△",E16="△"),"△ 着手済・要確認",IF(OR(D16="？",E16="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D16" s="13">
+        <f>IF(J16="計画なし","－",IF(J16="策定済","✕",IF(H16="","？",IF(AND(H16&gt;=TGT_MIN,H16&lt;=TGT_MAX),IF(J16="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E16" s="13">
+        <f>IF(P16="計画なし","－",IF(P16="策定済","✕",IF(N16="","？",IF(AND(N16&gt;=TGT_MIN,N16&lt;=TGT_MAX),IF(P16="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="n"/>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K16" s="11" t="n"/>
+      <c r="L16" s="11" t="n"/>
+      <c r="M16" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N16" s="13" t="n"/>
+      <c r="O16" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P16" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q16" s="11" t="n"/>
+      <c r="R16" s="11" t="inlineStr">
+        <is>
+          <t>交通：村独自計画は確認できず（村営路線なし、タクシー助成「しんタク」実証）。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：環境基本計画は村の個別計画ページで確認できず https://www.vill.shinto.gunma.jp/administration/000366/000378/index.html 。</t>
+        </is>
+      </c>
+      <c r="S16" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T16" s="11" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>吉岡町</t>
+        </is>
+      </c>
+      <c r="C17" s="12">
+        <f>IF(OR(D17="◎",E17="◎"),"◎ 営業",IF(OR(D17="△",E17="△"),"△ 着手済・要確認",IF(OR(D17="？",E17="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D17" s="13">
+        <f>IF(J17="計画なし","－",IF(J17="策定済","✕",IF(H17="","？",IF(AND(H17&gt;=TGT_MIN,H17&lt;=TGT_MAX),IF(J17="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E17" s="13">
+        <f>IF(P17="計画なし","－",IF(P17="策定済","✕",IF(N17="","？",IF(AND(N17&gt;=TGT_MIN,N17&lt;=TGT_MAX),IF(P17="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="n"/>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J17" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K17" s="11" t="n"/>
+      <c r="L17" s="11" t="n"/>
+      <c r="M17" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N17" s="13" t="n"/>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P17" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q17" s="11" t="n"/>
+      <c r="R17" s="11" t="inlineStr">
+        <is>
+          <t>交通：町独自計画は確認できず。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。環境：環境基本計画は確認できず（再生可能エネルギービジョン、事務事業編、R5.12ゼロカーボンシティ宣言 https://www.town.yoshioka.gunma.jp/kurashi/kankyo/post_163.html ）。</t>
+        </is>
+      </c>
+      <c r="S17" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T17" s="11" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>上野村</t>
+        </is>
+      </c>
+      <c r="C18" s="12">
+        <f>IF(OR(D18="◎",E18="◎"),"◎ 営業",IF(OR(D18="△",E18="△"),"△ 着手済・要確認",IF(OR(D18="？",E18="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D18" s="13">
+        <f>IF(J18="計画なし","－",IF(J18="策定済","✕",IF(H18="","？",IF(AND(H18&gt;=TGT_MIN,H18&lt;=TGT_MAX),IF(J18="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E18" s="13">
+        <f>IF(P18="計画なし","－",IF(P18="策定済","✕",IF(N18="","？",IF(AND(N18&gt;=TGT_MIN,N18&lt;=TGT_MAX),IF(P18="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="n"/>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K18" s="11" t="n"/>
+      <c r="L18" s="11" t="n"/>
+      <c r="M18" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N18" s="13" t="n"/>
+      <c r="O18" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P18" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q18" s="11" t="n"/>
+      <c r="R18" s="11" t="inlineStr">
+        <is>
+          <t>交通：村独自計画は確認できず（路線バス・乗合タクシー、村内循環EVデマンドバス。多野藤岡広域路線バス奥多野線）。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：環境基本計画は確認できず（地球温暖化対策実行計画R5.3、脱炭素先行地域計画、Ueno5つのゼロ宣言 https://www.uenomura.jp/admin/politics/post-30.html ）。</t>
+        </is>
+      </c>
+      <c r="S18" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T18" s="11" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>神流町</t>
+        </is>
+      </c>
+      <c r="C19" s="12">
+        <f>IF(OR(D19="◎",E19="◎"),"◎ 営業",IF(OR(D19="△",E19="△"),"△ 着手済・要確認",IF(OR(D19="？",E19="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D19" s="13">
+        <f>IF(J19="計画なし","－",IF(J19="策定済","✕",IF(H19="","？",IF(AND(H19&gt;=TGT_MIN,H19&lt;=TGT_MAX),IF(J19="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E19" s="13">
+        <f>IF(P19="計画なし","－",IF(P19="策定済","✕",IF(N19="","？",IF(AND(N19&gt;=TGT_MIN,N19&lt;=TGT_MAX),IF(P19="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F19" s="11" t="n"/>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K19" s="11" t="n"/>
+      <c r="L19" s="11" t="n"/>
+      <c r="M19" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N19" s="13" t="n"/>
+      <c r="O19" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P19" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q19" s="11" t="n"/>
+      <c r="R19" s="11" t="inlineStr">
+        <is>
+          <t>交通：町独自計画は確認できず（公共交通は多野藤岡広域市町村圏振興整備組合が所管）。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：環境基本計画は確認できず（環境政策ページ https://www.town.kanna.gunma.jp/gyouseijouhou/kouhyoujikou/883.html 、R2.7ゼロカーボンシティ宣言）。</t>
+        </is>
+      </c>
+      <c r="S19" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T19" s="11" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>下仁田町</t>
+        </is>
+      </c>
+      <c r="C20" s="12">
+        <f>IF(OR(D20="◎",E20="◎"),"◎ 営業",IF(OR(D20="△",E20="△"),"△ 着手済・要確認",IF(OR(D20="？",E20="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D20" s="13">
+        <f>IF(J20="計画なし","－",IF(J20="策定済","✕",IF(H20="","？",IF(AND(H20&gt;=TGT_MIN,H20&lt;=TGT_MAX),IF(J20="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E20" s="13">
+        <f>IF(P20="計画なし","－",IF(P20="策定済","✕",IF(N20="","？",IF(AND(N20&gt;=TGT_MIN,N20&lt;=TGT_MAX),IF(P20="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="n"/>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K20" s="11" t="n"/>
+      <c r="L20" s="11" t="inlineStr">
+        <is>
+          <t>第2次下仁田町環境基本計画</t>
+        </is>
+      </c>
+      <c r="M20" s="11" t="inlineStr">
+        <is>
+          <t>H29〜R8</t>
+        </is>
+      </c>
+      <c r="N20" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="O20" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P20" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="Q20" s="14" t="inlineStr">
+        <is>
+          <t>https://www.town.shimonita.lg.jp/hoken-kankyo/m01/m02/m01/kankyo-kihonplan.pdf</t>
+        </is>
+      </c>
+      <c r="R20" s="11" t="inlineStr">
+        <is>
+          <t>交通：町独自計画は確認できず（町営バス5路線、デマンド検討）。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：H29〜H38（R8）でR8年度終期、次期（第3次）計画の作業は検索で確認できず。要注視。</t>
+        </is>
+      </c>
+      <c r="S20" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T20" s="11" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>南牧村</t>
+        </is>
+      </c>
+      <c r="C21" s="12">
+        <f>IF(OR(D21="◎",E21="◎"),"◎ 営業",IF(OR(D21="△",E21="△"),"△ 着手済・要確認",IF(OR(D21="？",E21="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D21" s="13">
+        <f>IF(J21="計画なし","－",IF(J21="策定済","✕",IF(H21="","？",IF(AND(H21&gt;=TGT_MIN,H21&lt;=TGT_MAX),IF(J21="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E21" s="13">
+        <f>IF(P21="計画なし","－",IF(P21="策定済","✕",IF(N21="","？",IF(AND(N21&gt;=TGT_MIN,N21&lt;=TGT_MAX),IF(P21="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F21" s="11" t="n"/>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="n"/>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K21" s="11" t="n"/>
+      <c r="L21" s="11" t="n"/>
+      <c r="M21" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N21" s="13" t="n"/>
+      <c r="O21" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P21" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q21" s="11" t="n"/>
+      <c r="R21" s="11" t="inlineStr">
+        <is>
+          <t>交通：村独自計画は検索で確認できず。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：環境基本計画は確認できず。</t>
+        </is>
+      </c>
+      <c r="S21" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T21" s="11" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>甘楽町</t>
+        </is>
+      </c>
+      <c r="C22" s="12">
+        <f>IF(OR(D22="◎",E22="◎"),"◎ 営業",IF(OR(D22="△",E22="△"),"△ 着手済・要確認",IF(OR(D22="？",E22="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D22" s="13">
+        <f>IF(J22="計画なし","－",IF(J22="策定済","✕",IF(H22="","？",IF(AND(H22&gt;=TGT_MIN,H22&lt;=TGT_MAX),IF(J22="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E22" s="13">
+        <f>IF(P22="計画なし","－",IF(P22="策定済","✕",IF(N22="","？",IF(AND(N22&gt;=TGT_MIN,N22&lt;=TGT_MAX),IF(P22="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>甘楽町地域公共交通計画</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>R6〜R10</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="K22" s="14" t="inlineStr">
+        <is>
+          <t>https://www.town.kanra.lg.jp/kikaku/chousei/sozai/other/traffic_plan.pdf</t>
+        </is>
+      </c>
+      <c r="L22" s="11" t="n"/>
+      <c r="M22" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N22" s="13" t="n"/>
+      <c r="O22" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P22" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q22" s="11" t="n"/>
+      <c r="R22" s="11" t="inlineStr">
+        <is>
+          <t>交通：R6.4策定（甘楽町地域公共交通協議会）、2024〜2028年度。環境：環境基本計画は確認できず（総合計画内で環境施策）。</t>
+        </is>
+      </c>
+      <c r="S22" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T22" s="11" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>中之条町</t>
+        </is>
+      </c>
+      <c r="C23" s="12">
+        <f>IF(OR(D23="◎",E23="◎"),"◎ 営業",IF(OR(D23="△",E23="△"),"△ 着手済・要確認",IF(OR(D23="？",E23="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D23" s="13">
+        <f>IF(J23="計画なし","－",IF(J23="策定済","✕",IF(H23="","？",IF(AND(H23&gt;=TGT_MIN,H23&lt;=TGT_MAX),IF(J23="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E23" s="13">
+        <f>IF(P23="計画なし","－",IF(P23="策定済","✕",IF(N23="","？",IF(AND(N23&gt;=TGT_MIN,N23&lt;=TGT_MAX),IF(P23="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>中之条町地域公共交通計画</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>R8〜R12</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="J23" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="K23" s="14" t="inlineStr">
+        <is>
+          <t>https://www.town.nakanojo.gunma.jp/soshiki/4/14126.html</t>
+        </is>
+      </c>
+      <c r="L23" s="11" t="inlineStr">
+        <is>
+          <t>第二次中之条町環境基本計画</t>
+        </is>
+      </c>
+      <c r="M23" s="11" t="inlineStr">
+        <is>
+          <t>2019策定（期間不明）</t>
+        </is>
+      </c>
+      <c r="N23" s="13" t="n"/>
+      <c r="O23" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P23" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="Q23" s="14" t="inlineStr">
+        <is>
+          <t>https://www.town.nakanojo.gunma.jp/soshiki/4/1284.html</t>
+        </is>
+      </c>
+      <c r="R23" s="11" t="inlineStr">
+        <is>
+          <t>交通：R8〜R12、パブコメ後2026.5公表。環境：2019年策定（計画一覧ページで確認、期間未確認。10年ならR10頃終期）。</t>
+        </is>
+      </c>
+      <c r="S23" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T23" s="11" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>長野原町</t>
+        </is>
+      </c>
+      <c r="C24" s="12">
+        <f>IF(OR(D24="◎",E24="◎"),"◎ 営業",IF(OR(D24="△",E24="△"),"△ 着手済・要確認",IF(OR(D24="？",E24="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D24" s="13">
+        <f>IF(J24="計画なし","－",IF(J24="策定済","✕",IF(H24="","？",IF(AND(H24&gt;=TGT_MIN,H24&lt;=TGT_MAX),IF(J24="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E24" s="13">
+        <f>IF(P24="計画なし","－",IF(P24="策定済","✕",IF(N24="","？",IF(AND(N24&gt;=TGT_MIN,N24&lt;=TGT_MAX),IF(P24="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>長野原町地域公共交通計画</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="n"/>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="K24" s="14" t="inlineStr">
+        <is>
+          <t>https://www.town.naganohara.gunma.jp/www/contents/1681342705782/index.html</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="n"/>
+      <c r="M24" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N24" s="13" t="n"/>
+      <c r="O24" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P24" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q24" s="11" t="n"/>
+      <c r="R24" s="11" t="inlineStr">
+        <is>
+          <t>交通：R5頃策定（10〜20年後を見据える、R5年度から実現検討）。期間は検索で確認できず。JR吾妻線 長野原草津口〜大前間についてJR東日本が県・町・嬬恋村に交通体系の議論を申し入れ。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：環境基本計画は確認できず（地域新エネルギービジョンあり）。</t>
+        </is>
+      </c>
+      <c r="S24" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T24" s="11" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>嬬恋村</t>
+        </is>
+      </c>
+      <c r="C25" s="12">
+        <f>IF(OR(D25="◎",E25="◎"),"◎ 営業",IF(OR(D25="△",E25="△"),"△ 着手済・要確認",IF(OR(D25="？",E25="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D25" s="13">
+        <f>IF(J25="計画なし","－",IF(J25="策定済","✕",IF(H25="","？",IF(AND(H25&gt;=TGT_MIN,H25&lt;=TGT_MAX),IF(J25="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E25" s="13">
+        <f>IF(P25="計画なし","－",IF(P25="策定済","✕",IF(N25="","？",IF(AND(N25&gt;=TGT_MIN,N25&lt;=TGT_MAX),IF(P25="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F25" s="11" t="n"/>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="n"/>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K25" s="11" t="n"/>
+      <c r="L25" s="11" t="n"/>
+      <c r="M25" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N25" s="13" t="n"/>
+      <c r="O25" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P25" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q25" s="11" t="n"/>
+      <c r="R25" s="11" t="inlineStr">
+        <is>
+          <t>交通：村独自の地域公共交通計画は確認できず（総合計画後期R7〜R11で公共交通見直しを検討、デマンドバス）。JR吾妻線末端区間の在り方議論あり。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：環境基本計画は確認できず。</t>
+        </is>
+      </c>
+      <c r="S25" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T25" s="11" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>草津町</t>
+        </is>
+      </c>
+      <c r="C26" s="12">
+        <f>IF(OR(D26="◎",E26="◎"),"◎ 営業",IF(OR(D26="△",E26="△"),"△ 着手済・要確認",IF(OR(D26="？",E26="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D26" s="13">
+        <f>IF(J26="計画なし","－",IF(J26="策定済","✕",IF(H26="","？",IF(AND(H26&gt;=TGT_MIN,H26&lt;=TGT_MAX),IF(J26="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E26" s="13">
+        <f>IF(P26="計画なし","－",IF(P26="策定済","✕",IF(N26="","？",IF(AND(N26&gt;=TGT_MIN,N26&lt;=TGT_MAX),IF(P26="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F26" s="11" t="n"/>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H26" s="13" t="n"/>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J26" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K26" s="11" t="n"/>
+      <c r="L26" s="11" t="n"/>
+      <c r="M26" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N26" s="13" t="n"/>
+      <c r="O26" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P26" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q26" s="11" t="n"/>
+      <c r="R26" s="11" t="inlineStr">
+        <is>
+          <t>交通：町独自計画は確認できず（総合戦略で公共交通の充実が課題）。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：環境基本計画は確認できず。</t>
+        </is>
+      </c>
+      <c r="S26" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T26" s="11" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>高山村</t>
+        </is>
+      </c>
+      <c r="C27" s="12">
+        <f>IF(OR(D27="◎",E27="◎"),"◎ 営業",IF(OR(D27="△",E27="△"),"△ 着手済・要確認",IF(OR(D27="？",E27="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D27" s="13">
+        <f>IF(J27="計画なし","－",IF(J27="策定済","✕",IF(H27="","？",IF(AND(H27&gt;=TGT_MIN,H27&lt;=TGT_MAX),IF(J27="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E27" s="13">
+        <f>IF(P27="計画なし","－",IF(P27="策定済","✕",IF(N27="","？",IF(AND(N27&gt;=TGT_MIN,N27&lt;=TGT_MAX),IF(P27="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F27" s="11" t="n"/>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="n"/>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J27" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K27" s="11" t="n"/>
+      <c r="L27" s="11" t="n"/>
+      <c r="M27" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N27" s="13" t="n"/>
+      <c r="O27" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P27" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q27" s="11" t="n"/>
+      <c r="R27" s="11" t="inlineStr">
+        <is>
+          <t>交通：村独自計画は確認できず（路線バスのデマンド化・有償運送の方針、第6次総合計画R7〜R16）。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：環境基本計画は確認できず。</t>
+        </is>
+      </c>
+      <c r="S27" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T27" s="11" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>東吾妻町</t>
+        </is>
+      </c>
+      <c r="C28" s="12">
+        <f>IF(OR(D28="◎",E28="◎"),"◎ 営業",IF(OR(D28="△",E28="△"),"△ 着手済・要確認",IF(OR(D28="？",E28="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D28" s="13">
+        <f>IF(J28="計画なし","－",IF(J28="策定済","✕",IF(H28="","？",IF(AND(H28&gt;=TGT_MIN,H28&lt;=TGT_MAX),IF(J28="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E28" s="13">
+        <f>IF(P28="計画なし","－",IF(P28="策定済","✕",IF(N28="","？",IF(AND(N28&gt;=TGT_MIN,N28&lt;=TGT_MAX),IF(P28="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>東吾妻町地域公共交通計画</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>R4〜R8</t>
+        </is>
+      </c>
+      <c r="H28" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>着手済</t>
+        </is>
+      </c>
+      <c r="K28" s="14" t="inlineStr">
+        <is>
+          <t>https://www.town.higashiagatsuma.gunma.jp/www/contents/1650246606240/index.html</t>
+        </is>
+      </c>
+      <c r="L28" s="11" t="n"/>
+      <c r="M28" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N28" s="13" t="n"/>
+      <c r="O28" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P28" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q28" s="11" t="n"/>
+      <c r="R28" s="11" t="inlineStr">
+        <is>
+          <t>交通：2022〜2026年度でR8終期。2026.10.1付で「東吾妻町R9年度地域公共交通再編案」のパブコメを実施（町サイト新着、次期計画との関係は要確認）。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：環境基本計画は確認できず（地球温暖化対策実行計画のみ）。</t>
+        </is>
+      </c>
+      <c r="S28" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T28" s="11" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>片品村</t>
+        </is>
+      </c>
+      <c r="C29" s="12">
+        <f>IF(OR(D29="◎",E29="◎"),"◎ 営業",IF(OR(D29="△",E29="△"),"△ 着手済・要確認",IF(OR(D29="？",E29="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D29" s="13">
+        <f>IF(J29="計画なし","－",IF(J29="策定済","✕",IF(H29="","？",IF(AND(H29&gt;=TGT_MIN,H29&lt;=TGT_MAX),IF(J29="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E29" s="13">
+        <f>IF(P29="計画なし","－",IF(P29="策定済","✕",IF(N29="","？",IF(AND(N29&gt;=TGT_MIN,N29&lt;=TGT_MAX),IF(P29="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F29" s="11" t="n"/>
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="n"/>
+      <c r="I29" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J29" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K29" s="11" t="n"/>
+      <c r="L29" s="11" t="n"/>
+      <c r="M29" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N29" s="13" t="n"/>
+      <c r="O29" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P29" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q29" s="11" t="n"/>
+      <c r="R29" s="11" t="inlineStr">
+        <is>
+          <t>交通：村独自計画は確認できず（路線バスのみ、過疎計画R8〜R12、尾瀬の交通対策）。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：環境基本計画は確認できず（第5次総合計画R8〜R17内に環境保全）。</t>
+        </is>
+      </c>
+      <c r="S29" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T29" s="11" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>川場村</t>
+        </is>
+      </c>
+      <c r="C30" s="12">
+        <f>IF(OR(D30="◎",E30="◎"),"◎ 営業",IF(OR(D30="△",E30="△"),"△ 着手済・要確認",IF(OR(D30="？",E30="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D30" s="13">
+        <f>IF(J30="計画なし","－",IF(J30="策定済","✕",IF(H30="","？",IF(AND(H30&gt;=TGT_MIN,H30&lt;=TGT_MAX),IF(J30="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E30" s="13">
+        <f>IF(P30="計画なし","－",IF(P30="策定済","✕",IF(N30="","？",IF(AND(N30&gt;=TGT_MIN,N30&lt;=TGT_MAX),IF(P30="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F30" s="11" t="n"/>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H30" s="13" t="n"/>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J30" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K30" s="11" t="n"/>
+      <c r="L30" s="11" t="n"/>
+      <c r="M30" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N30" s="13" t="n"/>
+      <c r="O30" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P30" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q30" s="11" t="n"/>
+      <c r="R30" s="11" t="inlineStr">
+        <is>
+          <t>交通：村独自計画は確認できず。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：環境基本計画は確認できず。</t>
+        </is>
+      </c>
+      <c r="S30" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T30" s="11" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>昭和村</t>
+        </is>
+      </c>
+      <c r="C31" s="12">
+        <f>IF(OR(D31="◎",E31="◎"),"◎ 営業",IF(OR(D31="△",E31="△"),"△ 着手済・要確認",IF(OR(D31="？",E31="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D31" s="13">
+        <f>IF(J31="計画なし","－",IF(J31="策定済","✕",IF(H31="","？",IF(AND(H31&gt;=TGT_MIN,H31&lt;=TGT_MAX),IF(J31="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E31" s="13">
+        <f>IF(P31="計画なし","－",IF(P31="策定済","✕",IF(N31="","？",IF(AND(N31&gt;=TGT_MIN,N31&lt;=TGT_MAX),IF(P31="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F31" s="11" t="n"/>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H31" s="13" t="n"/>
+      <c r="I31" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J31" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K31" s="11" t="n"/>
+      <c r="L31" s="11" t="n"/>
+      <c r="M31" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N31" s="13" t="n"/>
+      <c r="O31" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P31" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q31" s="11" t="n"/>
+      <c r="R31" s="11" t="inlineStr">
+        <is>
+          <t>交通：村独自計画は確認できず。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：環境基本計画は確認できず。</t>
+        </is>
+      </c>
+      <c r="S31" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T31" s="11" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>みなかみ町</t>
+        </is>
+      </c>
+      <c r="C32" s="12">
+        <f>IF(OR(D32="◎",E32="◎"),"◎ 営業",IF(OR(D32="△",E32="△"),"△ 着手済・要確認",IF(OR(D32="？",E32="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D32" s="13">
+        <f>IF(J32="計画なし","－",IF(J32="策定済","✕",IF(H32="","？",IF(AND(H32&gt;=TGT_MIN,H32&lt;=TGT_MAX),IF(J32="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E32" s="13">
+        <f>IF(P32="計画なし","－",IF(P32="策定済","✕",IF(N32="","？",IF(AND(N32&gt;=TGT_MIN,N32&lt;=TGT_MAX),IF(P32="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F32" s="11" t="n"/>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H32" s="13" t="n"/>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J32" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K32" s="11" t="n"/>
+      <c r="L32" s="11" t="n"/>
+      <c r="M32" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N32" s="13" t="n"/>
+      <c r="O32" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P32" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q32" s="11" t="n"/>
+      <c r="R32" s="11" t="inlineStr">
+        <is>
+          <t>交通：町独自計画は確認できず。国交省資料に「みなかみ町でデータを基に地域公共交通計画の策定を行う」との記載あり https://www.mlit.go.jp/sogoseisaku/transport/content/001891615.pdf （策定予定の可能性）。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：環境基本計画は確認できず（SDGs未来都市計画あり）。</t>
+        </is>
+      </c>
+      <c r="S32" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T32" s="11" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>玉村町</t>
+        </is>
+      </c>
+      <c r="C33" s="12">
+        <f>IF(OR(D33="◎",E33="◎"),"◎ 営業",IF(OR(D33="△",E33="△"),"△ 着手済・要確認",IF(OR(D33="？",E33="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D33" s="13">
+        <f>IF(J33="計画なし","－",IF(J33="策定済","✕",IF(H33="","？",IF(AND(H33&gt;=TGT_MIN,H33&lt;=TGT_MAX),IF(J33="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E33" s="13">
+        <f>IF(P33="計画なし","－",IF(P33="策定済","✕",IF(N33="","？",IF(AND(N33&gt;=TGT_MIN,N33&lt;=TGT_MAX),IF(P33="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F33" s="11" t="n"/>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="n"/>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J33" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="K33" s="11" t="n"/>
+      <c r="L33" s="11" t="inlineStr">
+        <is>
+          <t>玉村町環境基本計画（2021-2030、後期計画R8.5公開）</t>
+        </is>
+      </c>
+      <c r="M33" s="11" t="inlineStr">
+        <is>
+          <t>R3〜R12</t>
+        </is>
+      </c>
+      <c r="N33" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="O33" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P33" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="Q33" s="14" t="inlineStr">
+        <is>
+          <t>https://www.town.tamamura.lg.jp/docs/2026050600012</t>
+        </is>
+      </c>
+      <c r="R33" s="11" t="inlineStr">
+        <is>
+          <t>交通：町独自の地域公共交通計画は確認できず。地域公共交通会議でR5年度に公共交通再編基本設計案 https://www.town.tamamura.lg.jp/docs/2023121400021/ 。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。環境：R3〜R12、後期計画を2026.5.7公開（R7.10アンケート実施）。</t>
+        </is>
+      </c>
+      <c r="S33" s="18" t="inlineStr">
+        <is>
+          <t>環境のみ調査</t>
+        </is>
+      </c>
+      <c r="T33" s="11" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>板倉町</t>
+        </is>
+      </c>
+      <c r="C34" s="12">
+        <f>IF(OR(D34="◎",E34="◎"),"◎ 営業",IF(OR(D34="△",E34="△"),"△ 着手済・要確認",IF(OR(D34="？",E34="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D34" s="13">
+        <f>IF(J34="計画なし","－",IF(J34="策定済","✕",IF(H34="","？",IF(AND(H34&gt;=TGT_MIN,H34&lt;=TGT_MAX),IF(J34="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E34" s="13">
+        <f>IF(P34="計画なし","－",IF(P34="策定済","✕",IF(N34="","？",IF(AND(N34&gt;=TGT_MIN,N34&lt;=TGT_MAX),IF(P34="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>第2次館林都市圏地域公共交通計画（1市4町共同）</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="inlineStr">
+        <is>
+          <t>R8〜R12</t>
+        </is>
+      </c>
+      <c r="H34" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>推定</t>
+        </is>
+      </c>
+      <c r="J34" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="K34" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.tatebayashi.gunma.jp/s015/shisei/040/020tatebayashitoshikenchiikikoukyoukoutukeikaku/2ndtatebayashitoshikentiikikoukyoukoutukeikaku.pdf</t>
+        </is>
+      </c>
+      <c r="L34" s="11" t="n"/>
+      <c r="M34" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N34" s="13" t="n"/>
+      <c r="O34" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P34" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q34" s="11" t="n"/>
+      <c r="R34" s="11" t="inlineStr">
+        <is>
+          <t>交通：第2次館林都市圏地域公共交通計画（館林市・板倉町・明和町・千代田町・邑楽町の1市4町共同）。前計画R3〜R7の後継、パブコメR7.12.22〜R8.1.16、目標年次R12（期間R8〜R12は推定）。環境：環境基本計画は町の計画一覧で確認できず https://www.town.itakura.gunma.jp/d000050/d000060/d000010/index.html 。</t>
+        </is>
+      </c>
+      <c r="S34" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T34" s="11" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>明和町</t>
+        </is>
+      </c>
+      <c r="C35" s="12">
+        <f>IF(OR(D35="◎",E35="◎"),"◎ 営業",IF(OR(D35="△",E35="△"),"△ 着手済・要確認",IF(OR(D35="？",E35="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D35" s="13">
+        <f>IF(J35="計画なし","－",IF(J35="策定済","✕",IF(H35="","？",IF(AND(H35&gt;=TGT_MIN,H35&lt;=TGT_MAX),IF(J35="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E35" s="13">
+        <f>IF(P35="計画なし","－",IF(P35="策定済","✕",IF(N35="","？",IF(AND(N35&gt;=TGT_MIN,N35&lt;=TGT_MAX),IF(P35="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
+          <t>第2次館林都市圏地域公共交通計画（1市4町共同）</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>R8〜R12</t>
+        </is>
+      </c>
+      <c r="H35" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>推定</t>
+        </is>
+      </c>
+      <c r="J35" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="K35" s="14" t="inlineStr">
+        <is>
+          <t>https://www.town.meiwa.gunma.jp/material/files/group/2/2ndkeikaku.pdf</t>
+        </is>
+      </c>
+      <c r="L35" s="11" t="n"/>
+      <c r="M35" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N35" s="13" t="n"/>
+      <c r="O35" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P35" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q35" s="11" t="n"/>
+      <c r="R35" s="11" t="inlineStr">
+        <is>
+          <t>交通：第2次館林都市圏地域公共交通計画（館林市・板倉町・明和町・千代田町・邑楽町の1市4町共同）。前計画R3〜R7の後継、パブコメR7.12.22〜R8.1.16、目標年次R12（期間R8〜R12は推定）。環境：環境基本計画は確認できず。</t>
+        </is>
+      </c>
+      <c r="S35" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T35" s="11" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>千代田町</t>
+        </is>
+      </c>
+      <c r="C36" s="12">
+        <f>IF(OR(D36="◎",E36="◎"),"◎ 営業",IF(OR(D36="△",E36="△"),"△ 着手済・要確認",IF(OR(D36="？",E36="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D36" s="13">
+        <f>IF(J36="計画なし","－",IF(J36="策定済","✕",IF(H36="","？",IF(AND(H36&gt;=TGT_MIN,H36&lt;=TGT_MAX),IF(J36="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E36" s="13">
+        <f>IF(P36="計画なし","－",IF(P36="策定済","✕",IF(N36="","？",IF(AND(N36&gt;=TGT_MIN,N36&lt;=TGT_MAX),IF(P36="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>第2次館林都市圏地域公共交通計画（1市4町共同）</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="inlineStr">
+        <is>
+          <t>R8〜R12</t>
+        </is>
+      </c>
+      <c r="H36" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>推定</t>
+        </is>
+      </c>
+      <c r="J36" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="K36" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.tatebayashi.gunma.jp/s015/shisei/040/020tatebayashitoshikenchiikikoukyoukoutukeikaku/2ndtatebayashitoshikentiikikoukyoukoutukeikaku.pdf</t>
+        </is>
+      </c>
+      <c r="L36" s="11" t="n"/>
+      <c r="M36" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="N36" s="13" t="n"/>
+      <c r="O36" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="P36" s="13" t="inlineStr">
+        <is>
+          <t>計画なし</t>
+        </is>
+      </c>
+      <c r="Q36" s="11" t="n"/>
+      <c r="R36" s="11" t="inlineStr">
+        <is>
+          <t>交通：第2次館林都市圏地域公共交通計画（館林市・板倉町・明和町・千代田町・邑楽町の1市4町共同）。前計画R3〜R7の後継、パブコメR7.12.22〜R8.1.16、目標年次R12（期間R8〜R12は推定）。大泉町と共同の地域公共交通会議も設置。環境：環境基本計画は確認できず（地球温暖化防止実行計画R3〜R12、ゼロカーボンシティ表明）。</t>
+        </is>
+      </c>
+      <c r="S36" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T36" s="11" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>大泉町</t>
+        </is>
+      </c>
+      <c r="C37" s="12">
+        <f>IF(OR(D37="◎",E37="◎"),"◎ 営業",IF(OR(D37="△",E37="△"),"△ 着手済・要確認",IF(OR(D37="？",E37="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D37" s="13">
+        <f>IF(J37="計画なし","－",IF(J37="策定済","✕",IF(H37="","？",IF(AND(H37&gt;=TGT_MIN,H37&lt;=TGT_MAX),IF(J37="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E37" s="13">
+        <f>IF(P37="計画なし","－",IF(P37="策定済","✕",IF(N37="","？",IF(AND(N37&gt;=TGT_MIN,N37&lt;=TGT_MAX),IF(P37="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t>大泉町地域公共交通計画（策定中）</t>
+        </is>
+      </c>
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="n"/>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="J37" s="13" t="inlineStr">
+        <is>
+          <t>着手済</t>
+        </is>
+      </c>
+      <c r="K37" s="11" t="n"/>
+      <c r="L37" s="11" t="inlineStr">
+        <is>
+          <t>大泉町環境基本計画</t>
+        </is>
+      </c>
+      <c r="M37" s="11" t="inlineStr">
+        <is>
+          <t>R6〜R12</t>
+        </is>
+      </c>
+      <c r="N37" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="O37" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P37" s="13" t="inlineStr">
+        <is>
+          <t>未確認</t>
+        </is>
+      </c>
+      <c r="Q37" s="14" t="inlineStr">
+        <is>
+          <t>https://www.town.oizumi.gunma.jp/s024/gyosei/010/010/050kankyokihonkeikaku/20240325132109.html</t>
+        </is>
+      </c>
+      <c r="R37" s="11" t="inlineStr">
+        <is>
+          <t>交通：現行計画は確認できず。町サイトに「大泉町地域公共交通計画策定業務プロポーザルの再実施について」掲載（4月3日付、年は未確認） https://www.town.oizumi.gunma.jp/li/gyosei/120/020/ 。大泉町・千代田町地域公共交通会議で広域バスあおぞら・デマンド「ほほえみ」運営。群馬県地域公共交通計画（群馬県交通まちづくり戦略の見直し、R5〜R9、県全域を4広域圏で記載） https://www.pref.gunma.jp/page/140624.html が県全域をカバー。県はR8.9.29に4広域圏別の計画改定業務プロポーザルを公告（履行期限R9.3.12） https://www.pref.gunma.jp/site/nyuusatsu/list135-773.html 。環境：R6〜R12。</t>
+        </is>
+      </c>
+      <c r="S37" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T37" s="11" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>邑楽町</t>
+        </is>
+      </c>
+      <c r="C38" s="12">
+        <f>IF(OR(D38="◎",E38="◎"),"◎ 営業",IF(OR(D38="△",E38="△"),"△ 着手済・要確認",IF(OR(D38="？",E38="？"),"？ 期間要確認","✕ 対象外")))</f>
+        <v/>
+      </c>
+      <c r="D38" s="13">
+        <f>IF(J38="計画なし","－",IF(J38="策定済","✕",IF(H38="","？",IF(AND(H38&gt;=TGT_MIN,H38&lt;=TGT_MAX),IF(J38="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="E38" s="13">
+        <f>IF(P38="計画なし","－",IF(P38="策定済","✕",IF(N38="","？",IF(AND(N38&gt;=TGT_MIN,N38&lt;=TGT_MAX),IF(P38="着手済","△","◎"),"✕"))))</f>
+        <v/>
+      </c>
+      <c r="F38" s="11" t="inlineStr">
+        <is>
+          <t>第2次館林都市圏地域公共交通計画（1市4町共同）</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="inlineStr">
+        <is>
+          <t>R8〜R12</t>
+        </is>
+      </c>
+      <c r="H38" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>推定</t>
+        </is>
+      </c>
+      <c r="J38" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="K38" s="14" t="inlineStr">
+        <is>
+          <t>https://www.city.tatebayashi.gunma.jp/s015/shisei/040/020tatebayashitoshikenchiikikoukyoukoutukeikaku/2ndtatebayashitoshikentiikikoukyoukoutukeikaku.pdf</t>
+        </is>
+      </c>
+      <c r="L38" s="11" t="inlineStr">
+        <is>
+          <t>邑楽町環境基本計画</t>
+        </is>
+      </c>
+      <c r="M38" s="11" t="inlineStr">
+        <is>
+          <t>R7〜R16</t>
+        </is>
+      </c>
+      <c r="N38" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="O38" s="13" t="inlineStr">
+        <is>
+          <t>確認済</t>
+        </is>
+      </c>
+      <c r="P38" s="13" t="inlineStr">
+        <is>
+          <t>策定済</t>
+        </is>
+      </c>
+      <c r="Q38" s="14" t="inlineStr">
+        <is>
+          <t>https://www.town.ora.gunma.jp/s017/020/100/700/env-basicplan.pdf</t>
+        </is>
+      </c>
+      <c r="R38" s="11" t="inlineStr">
+        <is>
+          <t>交通：第2次館林都市圏地域公共交通計画（館林市・板倉町・明和町・千代田町・邑楽町の1市4町共同）。前計画R3〜R7の後継、パブコメR7.12.22〜R8.1.16、目標年次R12（期間R8〜R12は推定）。環境：R7.3策定、R7〜R16（期間は素案で確認）。</t>
+        </is>
+      </c>
+      <c r="S38" s="15" t="inlineStr">
+        <is>
+          <t>調査済</t>
+        </is>
+      </c>
+      <c r="T38" s="11" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:T38"/>
+  <conditionalFormatting sqref="A4:T38">
+    <cfRule type="expression" priority="5" dxfId="0">
+      <formula>LEFT($C4,1)="◎"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="1">
+      <formula>LEFT($C4,1)="△"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="2">
+      <formula>LEFT($C4,1)="？"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="3">
+      <formula>LEFT($C4,1)="✕"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4:H38">
+    <cfRule type="expression" priority="1" dxfId="4" stopIfTrue="1">
+      <formula>AND(ISNUMBER(H4),H4&gt;=TGT_MIN,H4&lt;=TGT_MAX)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="5">
+      <formula>AND(ISNUMBER(H4),H4=TGT_MAX+1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N4:N38">
+    <cfRule type="expression" priority="3" dxfId="4" stopIfTrue="1">
+      <formula>AND(ISNUMBER(N4),N4&gt;=TGT_MIN,N4&lt;=TGT_MAX)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="5">
+      <formula>AND(ISNUMBER(N4),N4=TGT_MAX+1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="J4:J38 P4:P38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"未確認,着手済,策定済,計画なし"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId34"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5347,7 +8362,7 @@
       </c>
       <c r="R9" s="11" t="inlineStr">
         <is>
-          <t>交通：網形成計画（H30〜）をR6.3に地域公共交通計画として策定、計画期間は2018〜2027年度（R9終期）、2028年度以降に見直し予定。計画ページ https://www.city.kuji.lg.jp/soshiki/chiikizukurishinko/1/6/1/1835.html 。次期計画の委託等は未確認。三陸鉄道沿線地域等公共交通計画（岩手県・沿線12市町村の広域計画、2024策定） https://www.city.miyako.iwate.jp/gyosei/soshiki/kokyokotsuusuishin/2/1/605.html もカバー。環境：10年計画（R10以降に見直しとの記載あり）、正確な期間未確認。区域施策編改訂支援業務プロポーザルあり https://www.city.kuji.iwate.jp/assets/fukushi/siyousyo_ondankapropo.pdf 。 【ファクトチェック 2026-10-01: 確認できず】確認期間: None／次期: 確認できず／根拠: https://www.city.kuji.lg.jp/soshiki/chiikizukurishinko/1/6/1/1835.html 【追加調査 2026-10】【2026-10-02調査】検索3回で計画ページ https://www.city.kuji.lg.jp/soshiki/chiikizukurishinko/1/6/1/1835.html は確認できたが、計画期間（H30〜R9=2018〜2027年度）を示す本文抜粋は得られず推定のまま。市サイトはWebFetch不可（egress blocked）。次期計画の委託等も検索で見当たらず。 【追加調査 2026-10】環境：市サイト限定検索2回で『第1章 計画の基本的事項』(2021_kuji_kankyou_1.pdf)の本文として「2018年度から2027年度までの10年間」を確認（PDF直接取得は不可）。前回メモの『R10以降に見直し』と整合。R9終期のため次期（第3次）計画の策定委託・審議会・パブコメを検索したが見当たらず（着手未確認）。確認日2026-10-02。 根拠: 計画の期間は…2018年度から2027年度までの10年間とします</t>
+          <t>交通：網形成計画（H30〜）をR6.3に地域公共交通計画として策定、計画期間は2018〜2027年度（R9終期）とする検索結果が1回のみで、2026.10の再検索では裏付けが得られず推定、2028年度以降に見直し予定。計画ページ https://www.city.kuji.lg.jp/soshiki/chiikizukurishinko/1/6/1/1835.html 。次期計画の委託等は未確認。三陸鉄道沿線地域等公共交通計画（岩手県・沿線12市町村の広域計画、2024策定） https://www.city.miyako.iwate.jp/gyosei/soshiki/kokyokotsuusuishin/2/1/605.html もカバー。環境：10年計画（R10以降に見直しとの記載あり）、正確な期間未確認。区域施策編改訂支援業務プロポーザルあり https://www.city.kuji.iwate.jp/assets/fukushi/siyousyo_ondankapropo.pdf 。 【ファクトチェック 2026-10-01: 確認できず】確認期間: None／次期: 確認できず／根拠: https://www.city.kuji.lg.jp/soshiki/chiikizukurishinko/1/6/1/1835.html 【追加調査 2026-10】【2026-10-02調査】検索3回で計画ページ https://www.city.kuji.lg.jp/soshiki/chiikizukurishinko/1/6/1/1835.html は確認できたが、計画期間（H30〜R9=2018〜2027年度）を示す本文抜粋は得られず推定のまま。市サイトはWebFetch不可（egress blocked）。次期計画の委託等も検索で見当たらず。 【追加調査 2026-10】環境：市サイト限定検索2回で『第1章 計画の基本的事項』(2021_kuji_kankyou_1.pdf)の本文として「2018年度から2027年度までの10年間」を確認（PDF直接取得は不可）。前回メモの『R10以降に見直し』と整合。R9終期のため次期（第3次）計画の策定委託・審議会・パブコメを検索したが見当たらず（着手未確認）。確認日2026-10-02。 根拠: 計画の期間は…2018年度から2027年度までの10年間とします</t>
         </is>
       </c>
       <c r="S9" s="15" t="inlineStr">

</xml_diff>